<commit_message>
data: update 2026-09-08 [reports+xlsx]
</commit_message>
<xml_diff>
--- a/daily_logs/daily_2026-09-08.xlsx
+++ b/daily_logs/daily_2026-09-08.xlsx
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="E11" s="24" t="n">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
@@ -847,10 +847,10 @@
         </is>
       </c>
       <c r="E12" s="24" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
@@ -880,10 +880,10 @@
         </is>
       </c>
       <c r="E13" s="24" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
-          <t>Bull Stable</t>
+          <t>Bull Steepening</t>
         </is>
       </c>
       <c r="F14" s="24" t="n"/>
@@ -946,10 +946,10 @@
         </is>
       </c>
       <c r="E15" s="24" t="n">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F15" s="24" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="G15" s="6" t="n"/>
     </row>
@@ -975,10 +975,10 @@
         </is>
       </c>
       <c r="E16" s="24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G16" s="6" t="n"/>
     </row>
@@ -1035,10 +1035,10 @@
         </is>
       </c>
       <c r="E18" s="24" t="n">
-        <v>2.42</v>
+        <v>2.43</v>
       </c>
       <c r="F18" s="24" t="n">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="G18" s="6" t="n"/>
     </row>
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="E19" s="24" t="n">
-        <v>4.77</v>
+        <v>4.78</v>
       </c>
       <c r="F19" s="24" t="n">
-        <v>-8</v>
+        <v>-13</v>
       </c>
       <c r="G19" s="6" t="n"/>
     </row>
@@ -1093,10 +1093,10 @@
         </is>
       </c>
       <c r="E20" s="24" t="n">
-        <v>5.25</v>
+        <v>5.24</v>
       </c>
       <c r="F20" s="24" t="n">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="G20" s="6" t="n"/>
     </row>
@@ -1350,10 +1350,10 @@
         </is>
       </c>
       <c r="E29" s="24" t="n">
-        <v>2.35</v>
+        <v>2.37</v>
       </c>
       <c r="F29" s="24" t="n">
-        <v>-10</v>
+        <v>-8</v>
       </c>
       <c r="G29" s="6" t="n"/>
     </row>
@@ -1433,10 +1433,10 @@
         </is>
       </c>
       <c r="E32" s="24" t="n">
-        <v>2.33</v>
+        <v>2.34</v>
       </c>
       <c r="F32" s="24" t="n">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="G32" s="6" t="inlineStr">
         <is>
@@ -1621,10 +1621,10 @@
         </is>
       </c>
       <c r="E38" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F38" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G38" s="6" t="inlineStr">
         <is>
@@ -1687,10 +1687,10 @@
         </is>
       </c>
       <c r="E40" s="24" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G40" s="6" t="n"/>
     </row>
@@ -1772,10 +1772,10 @@
         </is>
       </c>
       <c r="E43" s="24" t="n">
-        <v>3.66</v>
+        <v>3.65</v>
       </c>
       <c r="F43" s="24" t="n">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="G43" s="6" t="n"/>
     </row>
@@ -2010,10 +2010,10 @@
         </is>
       </c>
       <c r="E51" s="24" t="n">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="F51" s="24" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
@@ -2221,10 +2221,10 @@
         </is>
       </c>
       <c r="E58" s="24" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F58" s="24" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
@@ -2914,8 +2914,8 @@
       <c r="E91" s="29" t="n"/>
       <c r="F91" s="21" t="inlineStr">
         <is>
-          <t>HY OAS 20dd=6.0bp [OK]
-HY OAS 5dd=-2.0bp
+          <t>HY OAS 20dd=2.0bp [OK]
+HY OAS 5dd=-5.0bp
 HYG 5d=-0.2% [OK]
 HYG DD%=None% max drawdown
 FXY 5d=2.5% [OK]

</xml_diff>